<commit_message>
reran consequence tables based on updated metrics
</commit_message>
<xml_diff>
--- a/wr_sdm/consequence_tables/weights.xlsx
+++ b/wr_sdm/consequence_tables/weights.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/consequence_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{34636CE1-49ED-4D4D-9578-10AA6B216942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2676C90D-9C9F-46CB-ADDE-52486684D771}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{34636CE1-49ED-4D4D-9578-10AA6B216942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D38C651-1EA5-4E61-B40A-E25987B57AF3}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="675" yWindow="3330" windowWidth="21600" windowHeight="11235" activeTab="1" xr2:uid="{9707D464-3622-4F04-9E64-EC8602A7C0C6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9707D464-3622-4F04-9E64-EC8602A7C0C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -123,13 +123,13 @@
     <t>mean_spawners_trib</t>
   </si>
   <si>
-    <t>mean_juv_rear_trib</t>
-  </si>
-  <si>
-    <t>num_trib</t>
-  </si>
-  <si>
     <t>ind_pop</t>
+  </si>
+  <si>
+    <t>mean_rear_prop</t>
+  </si>
+  <si>
+    <t>hab_access</t>
   </si>
 </sst>
 </file>
@@ -1397,13 +1397,13 @@
         <v>27</v>
       </c>
       <c r="L1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" t="s">
         <v>28</v>
-      </c>
-      <c r="M1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N1" t="s">
-        <v>30</v>
       </c>
       <c r="O1" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
updated documentation, weights columns
</commit_message>
<xml_diff>
--- a/wr_sdm/consequence_tables/weights.xlsx
+++ b/wr_sdm/consequence_tables/weights.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/consequence_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{34636CE1-49ED-4D4D-9578-10AA6B216942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D38C651-1EA5-4E61-B40A-E25987B57AF3}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{34636CE1-49ED-4D4D-9578-10AA6B216942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F1AB428-A4FD-4AE9-93E3-D0706EAC0B66}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9707D464-3622-4F04-9E64-EC8602A7C0C6}"/>
+    <workbookView xWindow="-24360" yWindow="-270" windowWidth="21600" windowHeight="11235" xr2:uid="{9707D464-3622-4F04-9E64-EC8602A7C0C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1361,6 +1361,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7CCEDC-F907-4EAF-BD51-4A41FE57A810}">
   <dimension ref="A1:T12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="9" max="9" width="27.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -1388,10 +1391,10 @@
         <v>24</v>
       </c>
       <c r="I1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" t="s">
         <v>25</v>
-      </c>
-      <c r="J1" t="s">
-        <v>26</v>
       </c>
       <c r="K1" t="s">
         <v>27</v>

</xml_diff>